<commit_message>
Remove references to the untracked dev/ notes
dev/ is git-ignored, so links and citations pointing into it did not
resolve for anyone cloning the repository.

- engine/README.md: point the R1-R14 matrix at datasets/common/review_rules.json
- output/firstVersion, output/thirdVersion READMEs: drop the citations;
  the rules they cited are already stated inline.
- engine/export_v3.py: the "cannot find is not none" basis text was written
  into 40 cells of the Form 3 basis sheet citing dev/03 - state the rule
  itself instead, and regenerate the thirdVersion workbooks.
- engine/poi_fetch.py: point at output/thirdVersion/README.md for the
  confidence tiers.
- README.md: drop the note in Notes about dev/ links not resolving.
</commit_message>
<xml_diff>
--- a/output/thirdVersion/表3_地價區段勘查表_已填.xlsx
+++ b/output/thirdVersion/表3_地價區段勘查表_已填.xlsx
@@ -20499,7 +20499,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>重要地標無『高鐵站』類型；新北市境內無高鐵站｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>重要地標無『高鐵站』類型；新北市境內無高鐵站｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -20623,7 +20623,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>無對應開放資料（公車站位屬站牌，不得代用）｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料（公車站位屬站牌，不得代用）｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -20665,7 +20665,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>樹林區 6 站全標示『施工中』，估價基準日 111.09.01 未通車，全數排除｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>樹林區 6 站全標示『施工中』，估價基準日 111.09.01 未通車，全數排除｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -21117,7 +21117,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>樹林區內 0 所；有效半徑 1,000m 內亦無鄰區大專院校｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>樹林區內 0 所；有效半徑 1,000m 內亦無鄰區大專院校｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -21569,7 +21569,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -22227,7 +22227,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>18 個來源皆無；改採 OSM｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>18 個來源皆無；改採 OSM｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -22393,7 +22393,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>土壤及地下水列管檔僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>土壤及地下水列管檔僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -22435,7 +22435,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -22559,7 +22559,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>土壤列管樹林區6筆僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>土壤列管樹林區6筆僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -22601,7 +22601,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>定義開放，無固定來源｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>定義開放，無固定來源｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -26328,7 +26328,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>重要地標無『高鐵站』類型；新北市境內無高鐵站｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>重要地標無『高鐵站』類型；新北市境內無高鐵站｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -26452,7 +26452,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>無對應開放資料（公車站位屬站牌，不得代用）｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料（公車站位屬站牌，不得代用）｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -26494,7 +26494,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>樹林區 6 站全標示『施工中』，估價基準日 111.09.01 未通車，全數排除｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>樹林區 6 站全標示『施工中』，估價基準日 111.09.01 未通車，全數排除｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -26946,7 +26946,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>樹林區內 0 所；有效半徑 1,000m 內亦無鄰區大專院校｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>樹林區內 0 所；有效半徑 1,000m 內亦無鄰區大專院校｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
@@ -27398,7 +27398,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
@@ -28056,7 +28056,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>18 個來源皆無；改採 OSM｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>18 個來源皆無；改採 OSM｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
@@ -28222,7 +28222,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>土壤及地下水列管檔僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>土壤及地下水列管檔僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
@@ -28264,7 +28264,7 @@
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
@@ -28388,7 +28388,7 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>土壤列管樹林區6筆僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>土壤列管樹林區6筆僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
@@ -28430,7 +28430,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>定義開放，無固定來源｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>定義開放，無固定來源｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>重要地標無『高鐵站』類型；新北市境內無高鐵站｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>重要地標無『高鐵站』類型；新北市境內無高鐵站｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
@@ -32281,7 +32281,7 @@
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>無對應開放資料（公車站位屬站牌，不得代用）｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料（公車站位屬站牌，不得代用）｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -32323,7 +32323,7 @@
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>樹林區 6 站全標示『施工中』，估價基準日 111.09.01 未通車，全數排除｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>樹林區 6 站全標示『施工中』，估價基準日 111.09.01 未通車，全數排除｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -32775,7 +32775,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>樹林區內 0 所；有效半徑 1,000m 內亦無鄰區大專院校｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>樹林區內 0 所；有效半徑 1,000m 內亦無鄰區大專院校｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -33227,7 +33227,7 @@
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G427" t="inlineStr">
@@ -33885,7 +33885,7 @@
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>18 個來源皆無；改採 OSM｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>18 個來源皆無；改採 OSM｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G443" t="inlineStr">
@@ -34051,7 +34051,7 @@
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>土壤及地下水列管檔僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>土壤及地下水列管檔僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G447" t="inlineStr">
@@ -34093,7 +34093,7 @@
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G448" t="inlineStr">
@@ -34217,7 +34217,7 @@
       </c>
       <c r="F451" t="inlineStr">
         <is>
-          <t>土壤列管樹林區6筆僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>土壤列管樹林區6筆僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G451" t="inlineStr">
@@ -34259,7 +34259,7 @@
       </c>
       <c r="F452" t="inlineStr">
         <is>
-          <t>定義開放，無固定來源｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>定義開放，無固定來源｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G452" t="inlineStr">
@@ -37986,7 +37986,7 @@
       </c>
       <c r="F547" t="inlineStr">
         <is>
-          <t>重要地標無『高鐵站』類型；新北市境內無高鐵站｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>重要地標無『高鐵站』類型；新北市境內無高鐵站｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G547" t="inlineStr">
@@ -38110,7 +38110,7 @@
       </c>
       <c r="F550" t="inlineStr">
         <is>
-          <t>無對應開放資料（公車站位屬站牌，不得代用）｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料（公車站位屬站牌，不得代用）｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G550" t="inlineStr">
@@ -38152,7 +38152,7 @@
       </c>
       <c r="F551" t="inlineStr">
         <is>
-          <t>樹林區 6 站全標示『施工中』，估價基準日 111.09.01 未通車，全數排除｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>樹林區 6 站全標示『施工中』，估價基準日 111.09.01 未通車，全數排除｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G551" t="inlineStr">
@@ -38604,7 +38604,7 @@
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>樹林區內 0 所；有效半徑 1,000m 內亦無鄰區大專院校｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>樹林區內 0 所；有效半徑 1,000m 內亦無鄰區大專院校｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G562" t="inlineStr">
@@ -39056,7 +39056,7 @@
       </c>
       <c r="F573" t="inlineStr">
         <is>
-          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G573" t="inlineStr">
@@ -39714,7 +39714,7 @@
       </c>
       <c r="F589" t="inlineStr">
         <is>
-          <t>18 個來源皆無；改採 OSM｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>18 個來源皆無；改採 OSM｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G589" t="inlineStr">
@@ -39880,7 +39880,7 @@
       </c>
       <c r="F593" t="inlineStr">
         <is>
-          <t>土壤及地下水列管檔僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>土壤及地下水列管檔僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G593" t="inlineStr">
@@ -39922,7 +39922,7 @@
       </c>
       <c r="F594" t="inlineStr">
         <is>
-          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>無對應開放資料｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G594" t="inlineStr">
@@ -40046,7 +40046,7 @@
       </c>
       <c r="F597" t="inlineStr">
         <is>
-          <t>土壤列管樹林區6筆僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>土壤列管樹林區6筆僅載地段地號，須地籍定位｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G597" t="inlineStr">
@@ -40088,7 +40088,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>定義開放，無固定來源｜查無資料 ≠ 無設施，不得填「無」（dev/03 §3.4(c)）</t>
+          <t>定義開放，無固定來源｜查無資料 ≠ 無設施，不得填「無」（正向設施之「無」＝最劣級，嫌惡設施之「無」＝最優級）</t>
         </is>
       </c>
       <c r="G598" t="inlineStr">

</xml_diff>